<commit_message>
Updated Excel file - August 21
</commit_message>
<xml_diff>
--- a/12619425.xlsx
+++ b/12619425.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D381E2F-EE8E-43DD-8E10-CAD3F3FDAF73}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9C894FF-DB6B-4C45-8A22-89997F51621A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -232,6 +232,18 @@
   </si>
   <si>
     <t>too many classes</t>
+  </si>
+  <si>
+    <t>tired</t>
+  </si>
+  <si>
+    <t>did laundry, cooking and house stuff</t>
+  </si>
+  <si>
+    <t>satisfied</t>
+  </si>
+  <si>
+    <t>went to jalander to get some stuff</t>
   </si>
 </sst>
 </file>
@@ -1148,49 +1160,97 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15" t="str">
+    <row r="9" spans="1:14" ht="30.75">
+      <c r="A9" s="13">
+        <v>46254</v>
+      </c>
+      <c r="B9" s="14">
+        <v>410</v>
+      </c>
+      <c r="C9" s="14">
+        <v>160</v>
+      </c>
+      <c r="D9" s="14">
+        <v>120</v>
+      </c>
+      <c r="E9" s="14">
+        <v>20</v>
+      </c>
+      <c r="F9" s="14">
+        <v>0</v>
+      </c>
+      <c r="G9" s="14">
+        <v>0</v>
+      </c>
+      <c r="H9" s="14">
+        <v>350</v>
+      </c>
+      <c r="I9" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="15" t="str">
+        <v>1060</v>
+      </c>
+      <c r="J9" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="17"/>
-    </row>
-    <row r="10" spans="1:14">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="15" t="str">
+        <v>380</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="30.75">
+      <c r="A10" s="13">
+        <v>46255</v>
+      </c>
+      <c r="B10" s="14">
+        <v>460</v>
+      </c>
+      <c r="C10" s="14">
+        <v>200</v>
+      </c>
+      <c r="D10" s="14">
+        <v>140</v>
+      </c>
+      <c r="E10" s="14">
+        <v>30</v>
+      </c>
+      <c r="F10" s="14">
+        <v>0</v>
+      </c>
+      <c r="G10" s="14">
+        <v>0</v>
+      </c>
+      <c r="H10" s="14">
+        <v>200</v>
+      </c>
+      <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J10" s="15" t="str">
+        <v>1030</v>
+      </c>
+      <c r="J10" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
-      <c r="N10" s="17"/>
+        <v>410</v>
+      </c>
+      <c r="K10" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L10" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N10" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="13"/>

</xml_diff>

<commit_message>
Update dataset August 23
</commit_message>
<xml_diff>
--- a/12619425.xlsx
+++ b/12619425.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9C894FF-DB6B-4C45-8A22-89997F51621A}"/>
+  <xr:revisionPtr revIDLastSave="94" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFA26660-6457-4ED8-BDEC-D0B50A67562A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="71">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -244,6 +244,15 @@
   </si>
   <si>
     <t>went to jalander to get some stuff</t>
+  </si>
+  <si>
+    <t>went to play football late at night</t>
+  </si>
+  <si>
+    <t>Neutral</t>
+  </si>
+  <si>
+    <t>worked on my typing skills and read an article</t>
   </si>
 </sst>
 </file>
@@ -1252,49 +1261,97 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15" t="str">
+    <row r="11" spans="1:14" ht="30.75">
+      <c r="A11" s="13">
+        <v>46256</v>
+      </c>
+      <c r="B11" s="14">
+        <v>400</v>
+      </c>
+      <c r="C11" s="14">
+        <v>120</v>
+      </c>
+      <c r="D11" s="14">
+        <v>90</v>
+      </c>
+      <c r="E11" s="14">
+        <v>120</v>
+      </c>
+      <c r="F11" s="14">
+        <v>0</v>
+      </c>
+      <c r="G11" s="14">
+        <v>0</v>
+      </c>
+      <c r="H11" s="14">
+        <v>280</v>
+      </c>
+      <c r="I11" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="15" t="str">
+        <v>1010</v>
+      </c>
+      <c r="J11" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="17"/>
-    </row>
-    <row r="12" spans="1:14">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+        <v>430</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="30.75">
+      <c r="A12" s="13">
+        <v>46256</v>
+      </c>
+      <c r="B12" s="14">
+        <v>420</v>
+      </c>
+      <c r="C12" s="14">
+        <v>40</v>
+      </c>
+      <c r="D12" s="14">
+        <v>220</v>
+      </c>
+      <c r="E12" s="14">
+        <v>60</v>
+      </c>
+      <c r="F12" s="14">
+        <v>0</v>
+      </c>
+      <c r="G12" s="14">
+        <v>0</v>
+      </c>
+      <c r="H12" s="14">
+        <v>340</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="17"/>
+        <v>360</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="13"/>
@@ -1384,7 +1441,7 @@
       <c r="M16" s="16"/>
       <c r="N16" s="17"/>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" ht="15">
       <c r="A17" s="13"/>
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>

</xml_diff>

<commit_message>
Update Data set August 26
</commit_message>
<xml_diff>
--- a/12619425.xlsx
+++ b/12619425.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="94" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFA26660-6457-4ED8-BDEC-D0B50A67562A}"/>
+  <xr:revisionPtr revIDLastSave="119" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A45D2A0-E80F-46AE-881E-69249DB99663}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="75">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -253,6 +253,18 @@
   </si>
   <si>
     <t>worked on my typing skills and read an article</t>
+  </si>
+  <si>
+    <t>played a tournament match</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Unsatisfied</t>
+  </si>
+  <si>
+    <t>tired from all the classes</t>
   </si>
 </sst>
 </file>
@@ -1353,49 +1365,97 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+    <row r="13" spans="1:14" ht="15">
+      <c r="A13" s="13">
+        <v>46257</v>
+      </c>
+      <c r="B13" s="14">
+        <v>360</v>
+      </c>
+      <c r="C13" s="14">
+        <v>240</v>
+      </c>
+      <c r="D13" s="14">
+        <v>60</v>
+      </c>
+      <c r="E13" s="14">
+        <v>45</v>
+      </c>
+      <c r="F13" s="14">
+        <v>6</v>
+      </c>
+      <c r="G13" s="14">
+        <v>6</v>
+      </c>
+      <c r="H13" s="14">
+        <v>230</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>941</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="17"/>
-    </row>
-    <row r="14" spans="1:14">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+        <v>499</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="15">
+      <c r="A14" s="13">
+        <v>46258</v>
+      </c>
+      <c r="B14" s="14">
+        <v>380</v>
+      </c>
+      <c r="C14" s="14">
+        <v>120</v>
+      </c>
+      <c r="D14" s="14">
+        <v>90</v>
+      </c>
+      <c r="E14" s="14">
+        <v>30</v>
+      </c>
+      <c r="F14" s="14">
+        <v>6</v>
+      </c>
+      <c r="G14" s="14">
+        <v>6</v>
+      </c>
+      <c r="H14" s="14">
+        <v>250</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>876</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="17"/>
+        <v>564</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="13"/>

</xml_diff>

<commit_message>
Update Data set August 29
</commit_message>
<xml_diff>
--- a/12619425.xlsx
+++ b/12619425.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776-26271\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A45D2A0-E80F-46AE-881E-69249DB99663}"/>
+  <xr:revisionPtr revIDLastSave="184" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEAFDF74-5DAB-41C3-BB5B-08FBDAB9929E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="78">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -252,9 +252,6 @@
     <t>Neutral</t>
   </si>
   <si>
-    <t>worked on my typing skills and read an article</t>
-  </si>
-  <si>
     <t>played a tournament match</t>
   </si>
   <si>
@@ -265,6 +262,18 @@
   </si>
   <si>
     <t>tired from all the classes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nothing much happenned </t>
+  </si>
+  <si>
+    <t>it rained like hell duirng the break</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iit was too hot </t>
+  </si>
+  <si>
+    <t xml:space="preserve">felt sleepy ui the classes </t>
   </si>
 </sst>
 </file>
@@ -1319,51 +1328,21 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="30.75">
-      <c r="A12" s="13">
-        <v>46256</v>
-      </c>
-      <c r="B12" s="14">
-        <v>420</v>
-      </c>
-      <c r="C12" s="14">
-        <v>40</v>
-      </c>
-      <c r="D12" s="14">
-        <v>220</v>
-      </c>
-      <c r="E12" s="14">
-        <v>60</v>
-      </c>
-      <c r="F12" s="14">
-        <v>0</v>
-      </c>
-      <c r="G12" s="14">
-        <v>0</v>
-      </c>
-      <c r="H12" s="14">
-        <v>340</v>
-      </c>
-      <c r="I12" s="15">
-        <f t="shared" si="0"/>
-        <v>1080</v>
-      </c>
-      <c r="J12" s="15">
-        <f t="shared" si="1"/>
-        <v>360</v>
-      </c>
-      <c r="K12" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="L12" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="M12" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="N12" s="17" t="s">
-        <v>70</v>
-      </c>
+    <row r="12" spans="1:14" ht="15">
+      <c r="A12" s="13"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="16"/>
+      <c r="N12" s="17"/>
     </row>
     <row r="13" spans="1:14" ht="15">
       <c r="A13" s="13">
@@ -1382,7 +1361,7 @@
         <v>45</v>
       </c>
       <c r="F13" s="14">
-        <v>6</v>
+        <v>350</v>
       </c>
       <c r="G13" s="14">
         <v>6</v>
@@ -1392,11 +1371,11 @@
       </c>
       <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v>941</v>
+        <v>1285</v>
       </c>
       <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v>499</v>
+        <v>155</v>
       </c>
       <c r="K13" s="16" t="s">
         <v>69</v>
@@ -1408,7 +1387,7 @@
         <v>55</v>
       </c>
       <c r="N13" s="17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="15">
@@ -1428,7 +1407,7 @@
         <v>30</v>
       </c>
       <c r="F14" s="14">
-        <v>6</v>
+        <v>350</v>
       </c>
       <c r="G14" s="14">
         <v>6</v>
@@ -1438,112 +1417,208 @@
       </c>
       <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v>876</v>
+        <v>1220</v>
       </c>
       <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v>564</v>
+        <v>220</v>
       </c>
       <c r="K14" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="L14" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="L14" s="16" t="s">
+      <c r="M14" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="N14" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="M14" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="N14" s="17" t="s">
+    </row>
+    <row r="15" spans="1:14" ht="15">
+      <c r="A15" s="13">
+        <v>46259</v>
+      </c>
+      <c r="B15" s="14">
+        <v>300</v>
+      </c>
+      <c r="C15" s="14">
+        <v>120</v>
+      </c>
+      <c r="D15" s="14">
+        <v>110</v>
+      </c>
+      <c r="E15" s="14">
+        <v>30</v>
+      </c>
+      <c r="F15" s="14">
+        <v>350</v>
+      </c>
+      <c r="G15" s="14">
+        <v>6</v>
+      </c>
+      <c r="H15" s="14">
+        <v>200</v>
+      </c>
+      <c r="I15" s="15">
+        <f t="shared" si="0"/>
+        <v>1110</v>
+      </c>
+      <c r="J15" s="15">
+        <f t="shared" si="1"/>
+        <v>330</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N15" s="17" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
-      <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="str">
+    <row r="16" spans="1:14" ht="30.75">
+      <c r="A16" s="13">
+        <v>46260</v>
+      </c>
+      <c r="B16" s="14">
+        <v>320</v>
+      </c>
+      <c r="C16" s="14">
+        <v>100</v>
+      </c>
+      <c r="D16" s="14">
+        <v>220</v>
+      </c>
+      <c r="E16" s="14">
+        <v>40</v>
+      </c>
+      <c r="F16" s="14">
+        <v>350</v>
+      </c>
+      <c r="G16" s="14">
+        <v>6</v>
+      </c>
+      <c r="H16" s="14">
+        <v>150</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
+        <v>1180</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="17"/>
-    </row>
-    <row r="16" spans="1:14">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
+        <v>260</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N16" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="15">
+      <c r="A17" s="13">
+        <v>46261</v>
+      </c>
+      <c r="B17" s="14">
+        <v>340</v>
+      </c>
+      <c r="C17" s="14">
+        <v>130</v>
+      </c>
+      <c r="D17" s="14">
+        <v>100</v>
+      </c>
+      <c r="E17" s="14">
+        <v>50</v>
+      </c>
+      <c r="F17" s="14">
+        <v>300</v>
+      </c>
+      <c r="G17" s="14">
+        <v>5</v>
+      </c>
+      <c r="H17" s="14">
+        <v>200</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
+        <v>1120</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="17"/>
-    </row>
-    <row r="17" spans="1:14" ht="15">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="str">
+        <v>320</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="15">
+      <c r="A18" s="13">
+        <v>46262</v>
+      </c>
+      <c r="B18" s="14">
+        <v>290</v>
+      </c>
+      <c r="C18" s="14">
+        <v>60</v>
+      </c>
+      <c r="D18" s="14">
+        <v>60</v>
+      </c>
+      <c r="E18" s="14">
+        <v>30</v>
+      </c>
+      <c r="F18" s="14">
+        <v>150</v>
+      </c>
+      <c r="G18" s="14">
+        <v>3</v>
+      </c>
+      <c r="H18" s="14">
+        <v>200</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
+        <v>790</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
-      <c r="N17" s="17"/>
-    </row>
-    <row r="18" spans="1:14">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
+        <v>650</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="13"/>

</xml_diff>